<commit_message>
Add earthworks Stage1 Google review flow
</commit_message>
<xml_diff>
--- a/output/price_registry_filled_v3.xlsx
+++ b/output/price_registry_filled_v3.xlsx
@@ -1425,7 +1425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H500"/>
+  <dimension ref="A1:H183"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.2"/>
   <cols>
     <col width="18.1111111111111" customWidth="1" min="1" max="1"/>
@@ -1504,7 +1504,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Поставщик: Оникс Бетон</t>
+          <t>Поставщик: Оникс Бетон Вариант поставщика/зоны. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для бетона, доставки и насоса.</t>
         </is>
       </c>
     </row>
@@ -1537,7 +1537,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Поставщик: Оникс Бетон</t>
+          <t>Поставщик: Оникс Бетон Вариант поставщика/зоны. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для бетона, доставки и насоса.</t>
         </is>
       </c>
     </row>
@@ -1565,7 +1565,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Поставщик: Оникс Бетон</t>
+          <t>Поставщик: Оникс Бетон Вариант поставщика/зоны. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для бетона, доставки и насоса.</t>
         </is>
       </c>
     </row>
@@ -1593,7 +1593,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Поставщик: Росбетон</t>
+          <t>Поставщик: Росбетон Вариант поставщика/зоны. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для бетона, доставки и насоса.</t>
         </is>
       </c>
     </row>
@@ -1626,7 +1626,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Поставщик: Росбетон</t>
+          <t>Поставщик: Росбетон Вариант поставщика/зоны. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для бетона, доставки и насоса.</t>
         </is>
       </c>
     </row>
@@ -1654,7 +1654,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Поставщик: Росбетон</t>
+          <t>Поставщик: Росбетон Вариант поставщика/зоны. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для бетона, доставки и насоса.</t>
         </is>
       </c>
     </row>
@@ -1680,7 +1680,7 @@
       <c r="F8" s="32" t="n"/>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Поставщик: РБУ 1</t>
+          <t>Поставщик: РБУ 1 Вариант поставщика/зоны. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для бетона, доставки и насоса.</t>
         </is>
       </c>
     </row>
@@ -1711,7 +1711,7 @@
       <c r="F9" s="32" t="n"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Поставщик: РБУ 1</t>
+          <t>Поставщик: РБУ 1 Вариант поставщика/зоны. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для бетона, доставки и насоса.</t>
         </is>
       </c>
     </row>
@@ -1737,7 +1737,7 @@
       <c r="F10" s="32" t="n"/>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Поставщик: РБУ 1</t>
+          <t>Поставщик: РБУ 1 Вариант поставщика/зоны. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для бетона, доставки и насоса.</t>
         </is>
       </c>
     </row>
@@ -1765,7 +1765,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Поставщик: Забетоном</t>
+          <t>Поставщик: Забетоном Вариант поставщика/зоны. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для бетона, доставки и насоса.</t>
         </is>
       </c>
     </row>
@@ -1798,7 +1798,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Поставщик: Забетоном</t>
+          <t>Поставщик: Забетоном Вариант поставщика/зоны. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для бетона, доставки и насоса.</t>
         </is>
       </c>
     </row>
@@ -1826,7 +1826,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Поставщик: Забетоном</t>
+          <t>Поставщик: Забетоном Вариант поставщика/зоны. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для бетона, доставки и насоса.</t>
         </is>
       </c>
     </row>
@@ -1852,7 +1852,7 @@
       <c r="F14" s="32" t="n"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Поставщик: Куб</t>
+          <t>Поставщик: Куб Вариант поставщика/зоны. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для бетона, доставки и насоса.</t>
         </is>
       </c>
     </row>
@@ -1883,7 +1883,7 @@
       <c r="F15" s="32" t="n"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Поставщик: Куб</t>
+          <t>Поставщик: Куб Вариант поставщика/зоны. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для бетона, доставки и насоса.</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
       <c r="F16" s="32" t="n"/>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Поставщик: Куб</t>
+          <t>Поставщик: Куб Вариант поставщика/зоны. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для бетона, доставки и насоса.</t>
         </is>
       </c>
     </row>
@@ -1935,7 +1935,7 @@
       <c r="F17" s="32" t="n"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Поставщик: Гранд бетон/Гарант бетон</t>
+          <t>Поставщик: Гранд бетон/Гарант бетон Вариант поставщика/зоны. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для бетона, доставки и насоса.</t>
         </is>
       </c>
     </row>
@@ -1966,7 +1966,7 @@
       <c r="F18" s="32" t="n"/>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Поставщик: Гранд бетон/Гарант бетон</t>
+          <t>Поставщик: Гранд бетон/Гарант бетон Вариант поставщика/зоны. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для бетона, доставки и насоса.</t>
         </is>
       </c>
     </row>
@@ -1992,7 +1992,7 @@
       <c r="F19" s="32" t="n"/>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Поставщик: Гранд бетон/Гарант бетон</t>
+          <t>Поставщик: Гранд бетон/Гарант бетон Вариант поставщика/зоны. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для бетона, доставки и насоса.</t>
         </is>
       </c>
     </row>
@@ -2018,7 +2018,7 @@
       <c r="F20" s="32" t="n"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Поставщик: Гарант бетон/Гранд бетон</t>
+          <t>Поставщик: Гарант бетон/Гранд бетон Вариант поставщика/зоны. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для бетона, доставки и насоса.</t>
         </is>
       </c>
     </row>
@@ -2049,7 +2049,7 @@
       <c r="F21" s="32" t="n"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Поставщик: Гарант бетон/Гранд бетон</t>
+          <t>Поставщик: Гарант бетон/Гранд бетон Вариант поставщика/зоны. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для бетона, доставки и насоса.</t>
         </is>
       </c>
     </row>
@@ -2075,7 +2075,7 @@
       <c r="F22" s="32" t="n"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Поставщик: Гарант бетон/Гранд бетон</t>
+          <t>Поставщик: Гарант бетон/Гранд бетон Вариант поставщика/зоны. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для бетона, доставки и насоса.</t>
         </is>
       </c>
     </row>
@@ -2101,7 +2101,7 @@
       <c r="F23" s="32" t="n"/>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Поставщик: МЖБК/Забетоном</t>
+          <t>Поставщик: МЖБК/Забетоном Вариант поставщика/зоны. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для бетона, доставки и насоса.</t>
         </is>
       </c>
     </row>
@@ -2132,7 +2132,7 @@
       <c r="F24" s="32" t="n"/>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Поставщик: МЖБК/Забетоном</t>
+          <t>Поставщик: МЖБК/Забетоном Вариант поставщика/зоны. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для бетона, доставки и насоса.</t>
         </is>
       </c>
     </row>
@@ -2158,7 +2158,7 @@
       <c r="F25" s="32" t="n"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Поставщик: МЖБК/Забетоном</t>
+          <t>Поставщик: МЖБК/Забетоном Вариант поставщика/зоны. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для бетона, доставки и насоса.</t>
         </is>
       </c>
     </row>
@@ -2187,6 +2187,11 @@
         <v>1400</v>
       </c>
       <c r="F26" s="32" t="n"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Вариант поставки по зоне. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для sand_m3.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2213,6 +2218,11 @@
         <v>1300</v>
       </c>
       <c r="F27" s="32" t="n"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Вариант поставки по зоне. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для sand_m3.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2239,6 +2249,11 @@
         <v>1300</v>
       </c>
       <c r="F28" s="32" t="n"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Вариант поставки по зоне. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для sand_m3.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2265,6 +2280,11 @@
         <v>1300</v>
       </c>
       <c r="F29" s="32" t="n"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Вариант поставки по зоне. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для sand_m3.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2291,6 +2311,11 @@
         <v>1300</v>
       </c>
       <c r="F30" s="32" t="n"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Вариант поставки по зоне. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для sand_m3.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2317,6 +2342,11 @@
         <v>1300</v>
       </c>
       <c r="F31" s="32" t="n"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Вариант поставки по зоне. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для sand_m3.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2343,6 +2373,11 @@
         <v>1300</v>
       </c>
       <c r="F32" s="32" t="n"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Вариант поставки по зоне. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для sand_m3.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2369,6 +2404,11 @@
         <v>1300</v>
       </c>
       <c r="F33" s="32" t="n"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Вариант поставки по зоне. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для sand_m3.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2395,6 +2435,11 @@
         <v>1300</v>
       </c>
       <c r="F34" s="32" t="n"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Вариант поставки по зоне. price_code не проставлен автоматически: нужно правило выбора зоны/поставщика для sand_m3.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2418,6 +2463,11 @@
       <c r="F35" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2441,6 +2491,11 @@
       <c r="F36" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2464,6 +2519,11 @@
       <c r="F37" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2487,6 +2547,11 @@
       <c r="F38" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2510,6 +2575,11 @@
       <c r="F39" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2533,6 +2603,11 @@
       <c r="F40" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2556,6 +2631,11 @@
       <c r="F41" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2579,6 +2659,11 @@
       <c r="F42" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2602,6 +2687,11 @@
       <c r="F43" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2625,6 +2715,11 @@
       <c r="F44" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2648,6 +2743,11 @@
       <c r="F45" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2671,6 +2771,11 @@
       <c r="F46" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2694,6 +2799,11 @@
       <c r="F47" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2717,6 +2827,11 @@
       <c r="F48" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2740,6 +2855,11 @@
       <c r="F49" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2763,6 +2883,11 @@
       <c r="F50" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2786,6 +2911,11 @@
       <c r="F51" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2809,6 +2939,11 @@
       <c r="F52" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2832,6 +2967,11 @@
       <c r="F53" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2855,6 +2995,11 @@
       <c r="F54" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2878,6 +3023,11 @@
       <c r="F55" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2901,6 +3051,16 @@
       <c r="F56" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>price_code проставлен автоматически по точному совпадению номенклатуры; проверьте цену/единицу.</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>plywood_1520x1520_18mm_sheet</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2924,6 +3084,11 @@
       <c r="F57" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2947,6 +3112,11 @@
       <c r="F58" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2970,6 +3140,11 @@
       <c r="F59" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2993,6 +3168,11 @@
       <c r="F60" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -3016,6 +3196,11 @@
       <c r="F61" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3039,6 +3224,11 @@
       <c r="F62" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3062,6 +3252,11 @@
       <c r="F63" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3085,6 +3280,11 @@
       <c r="F64" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3108,6 +3308,11 @@
       <c r="F65" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3131,6 +3336,11 @@
       <c r="F66" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3154,6 +3364,11 @@
       <c r="F67" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -3177,6 +3392,11 @@
       <c r="F68" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -3200,6 +3420,11 @@
       <c r="F69" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -3223,6 +3448,11 @@
       <c r="F70" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -3246,6 +3476,11 @@
       <c r="F71" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -3269,6 +3504,11 @@
       <c r="F72" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -3292,6 +3532,11 @@
       <c r="F73" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -3315,6 +3560,11 @@
       <c r="F74" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -3338,6 +3588,11 @@
       <c r="F75" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -3361,6 +3616,11 @@
       <c r="F76" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3384,6 +3644,11 @@
       <c r="F77" s="32" t="n">
         <v>46154</v>
       </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Каталожная позиция поставщика. price_code добавляется только если калькулятор ссылается на эту конкретную номенклатуру.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3410,6 +3675,16 @@
       <c r="F78" s="32" t="n">
         <v>46146</v>
       </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>price_code проставлен автоматически по точному совпадению номенклатуры; проверьте цену/единицу.</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>block_adhesive_bag</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3440,7 +3715,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>с 15.05; Вместимость в машину: 34,56 м3</t>
+          <t>с 15.05; Вместимость в машину: 34,56 м3 Каталожная/поставщическая позиция. price_code не проставлен автоматически, если нет однозначной связи с текущей строкой калькулятора.</t>
         </is>
       </c>
     </row>
@@ -3473,7 +3748,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>С 15.05; Вместимость в машину: 32,4 м3</t>
+          <t>С 15.05; Вместимость в машину: 32,4 м3 Каталожная/поставщическая позиция. price_code не проставлен автоматически, если нет однозначной связи с текущей строкой калькулятора.</t>
         </is>
       </c>
     </row>
@@ -3504,6 +3779,11 @@
       <c r="F81" s="32" t="n">
         <v>46146</v>
       </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Каталожная/поставщическая позиция. price_code не проставлен автоматически, если нет однозначной связи с текущей строкой калькулятора.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -3532,6 +3812,11 @@
       <c r="F82" s="32" t="n">
         <v>46146</v>
       </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Каталожная/поставщическая позиция. price_code не проставлен автоматически, если нет однозначной связи с текущей строкой калькулятора.</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -3558,6 +3843,12 @@
       <c r="F83" s="32" t="n">
         <v>46146</v>
       </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>price_code проставлен автоматически по точному совпадению номенклатуры; проверьте цену/единицу. Каталожная/поставщическая позиция. price_code не проставлен автоматически, если нет однозначной связи с текущей строкой калькулятора.</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -3584,6 +3875,11 @@
       <c r="F84" s="32" t="n">
         <v>46146</v>
       </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Каталожная/поставщическая позиция. price_code не проставлен автоматически, если нет однозначной связи с текущей строкой калькулятора.</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -3610,6 +3906,11 @@
       <c r="F85" s="32" t="n">
         <v>46146</v>
       </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Каталожная/поставщическая позиция. price_code не проставлен автоматически, если нет однозначной связи с текущей строкой калькулятора.</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -3638,7 +3939,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Вместимость в машину: 2640</t>
+          <t>Вместимость в машину: 2640 Каталожная/поставщическая позиция. price_code не проставлен автоматически, если нет однозначной связи с текущей строкой калькулятора.</t>
         </is>
       </c>
     </row>
@@ -3669,7 +3970,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Вместимость в машину: 1760</t>
+          <t>Вместимость в машину: 1760 Каталожная/поставщическая позиция. price_code не проставлен автоматически, если нет однозначной связи с текущей строкой калькулятора.</t>
         </is>
       </c>
     </row>
@@ -3700,7 +4001,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Вместимость в машину: 1368</t>
+          <t>Вместимость в машину: 1368 Каталожная/поставщическая позиция. price_code не проставлен автоматически, если нет однозначной связи с текущей строкой калькулятора.</t>
         </is>
       </c>
     </row>
@@ -3731,7 +4032,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Вместимость в машину: 1320</t>
+          <t>Вместимость в машину: 1320 Каталожная/поставщическая позиция. price_code не проставлен автоматически, если нет однозначной связи с текущей строкой калькулятора.</t>
         </is>
       </c>
     </row>
@@ -3762,7 +4063,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Вместимость в машину: 1320</t>
+          <t>Вместимость в машину: 1320 Каталожная/поставщическая позиция. price_code не проставлен автоматически, если нет однозначной связи с текущей строкой калькулятора.</t>
         </is>
       </c>
     </row>
@@ -3793,7 +4094,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Вместимость в машину: 1320</t>
+          <t>Вместимость в машину: 1320 Каталожная/поставщическая позиция. price_code не проставлен автоматически, если нет однозначной связи с текущей строкой калькулятора.</t>
         </is>
       </c>
     </row>
@@ -3824,7 +4125,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Вместимость в машину: 1100</t>
+          <t>Вместимость в машину: 1100 Каталожная/поставщическая позиция. price_code не проставлен автоматически, если нет однозначной связи с текущей строкой калькулятора.</t>
         </is>
       </c>
     </row>
@@ -3855,7 +4156,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Вместимость в машину: 1100</t>
+          <t>Вместимость в машину: 1100 Каталожная/поставщическая позиция. price_code не проставлен автоматически, если нет однозначной связи с текущей строкой калькулятора.</t>
         </is>
       </c>
     </row>
@@ -3886,7 +4187,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Вместимость в машину: h=330мм, габариты 200×250мм, вес 13кг, 63 шт на поддоне</t>
+          <t>Вместимость в машину: h=330мм, габариты 200×250мм, вес 13кг, 63 шт на поддоне Каталожная/поставщическая позиция. price_code не проставлен автоматически, если нет однозначной связи с текущей строкой калькулятора.</t>
         </is>
       </c>
     </row>
@@ -3989,7 +4290,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Вместимость в машину: h=330мм, габариты 500×360мм, вес 38кг, 16 шт на поддоне</t>
+          <t>Вместимость в машину: h=330мм, габариты 500×360мм, вес 38кг, 16 шт на поддоне Каталожная/поставщическая позиция. price_code не проставлен автоматически, если нет однозначной связи с текущей строкой калькулятора.</t>
         </is>
       </c>
     </row>
@@ -4018,6 +4319,11 @@
       <c r="F98" s="32" t="n">
         <v>46146</v>
       </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Каталожная/поставщическая позиция. price_code не проставлен автоматически, если нет однозначной связи с текущей строкой калькулятора.</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -4044,6 +4350,11 @@
       <c r="F99" s="32" t="n">
         <v>46146</v>
       </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Каталожная/поставщическая позиция. price_code не проставлен автоматически, если нет однозначной связи с текущей строкой калькулятора.</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -4101,6 +4412,11 @@
       <c r="F101" s="32" t="n">
         <v>46214</v>
       </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>price_code пока не сопоставлен; требуется ручная проверка связи с калькулятором.</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -4280,6 +4596,11 @@
         <v>75</v>
       </c>
       <c r="F107" s="32" t="n"/>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>price_code пока не сопоставлен; требуется ручная проверка связи с калькулятором.</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -4506,21 +4827,21 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Геотекстиль Дорнит 300 г.м2 (100м2) -1шт</t>
+          <t>Геотекстиль Дорнит 300 г.м2 (100м2)</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>рул</t>
+          <t>м2</t>
         </is>
       </c>
       <c r="E115" s="29" t="n">
-        <v>4562</v>
+        <v>109</v>
       </c>
       <c r="F115" s="32" t="n"/>
       <c r="G115" t="inlineStr">
         <is>
-          <t>Обновлено 04.05</t>
+          <t>Цена приведена к единице калькулятора: м2; ранее в прайсе была строка за рулон.</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
@@ -4549,6 +4870,11 @@
         <v>6610</v>
       </c>
       <c r="F116" s="32" t="n"/>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Позиция кровельного прайса. price_code не проставлен автоматически, если текущие калькуляторы пока не используют эту строку напрямую.</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -4570,6 +4896,12 @@
         <v>450</v>
       </c>
       <c r="F117" s="32" t="n"/>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>price_code проставлен автоматически по точному совпадению номенклатуры; проверьте цену/единицу. Позиция кровельного прайса. price_code не проставлен автоматически, если текущие калькуляторы пока не используют эту строку напрямую.</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -4617,6 +4949,16 @@
         <v>7377.89</v>
       </c>
       <c r="F119" s="32" t="n"/>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>price_code проставлен автоматически по точному совпадению номенклатуры; проверьте цену/единицу.</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>roof_eps100_technonikol_carbon_eco_m3</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -4638,6 +4980,16 @@
         <v>7155.34</v>
       </c>
       <c r="F120" s="32" t="n"/>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>price_code проставлен автоматически по точному совпадению номенклатуры; проверьте цену/единицу.</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>roof_eps50_technonikol_carbon_eco_m3</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -4659,6 +5011,16 @@
         <v>9888.67</v>
       </c>
       <c r="F121" s="32" t="n"/>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>price_code проставлен автоматически по точному совпадению номенклатуры; проверьте цену/единицу.</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>roof_eps_slope_2_1_plate_a_m3</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -4680,6 +5042,16 @@
         <v>9888.67</v>
       </c>
       <c r="F122" s="32" t="n"/>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>price_code проставлен автоматически по точному совпадению номенклатуры; проверьте цену/единицу.</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>roof_eps_slope_2_1_plate_b_m3</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -4701,6 +5073,16 @@
         <v>9888.67</v>
       </c>
       <c r="F123" s="32" t="n"/>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>price_code проставлен автоматически по точному совпадению номенклатуры; проверьте цену/единицу.</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>roof_eps_slope_4_2_plate_j_m3</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -4722,6 +5104,16 @@
         <v>9888.67</v>
       </c>
       <c r="F124" s="32" t="n"/>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>price_code проставлен автоматически по точному совпадению номенклатуры; проверьте цену/единицу.</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>roof_eps_slope_4_2_plate_k_m3</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -4743,6 +5135,11 @@
         <v>59.55</v>
       </c>
       <c r="F125" s="32" t="n"/>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Позиция кровельного прайса. price_code не проставлен автоматически, если текущие калькуляторы пока не используют эту строку напрямую.</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -4764,6 +5161,16 @@
         <v>57.56</v>
       </c>
       <c r="F126" s="32" t="n"/>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>price_code проставлен автоматически по точному совпадению номенклатуры; проверьте цену/единицу.</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>roof_geotextile_technonikol_prof_150_m2</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -4785,6 +5192,16 @@
         <v>90</v>
       </c>
       <c r="F127" s="32" t="n"/>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>price_code проставлен автоматически по точному совпадению номенклатуры; проверьте цену/единицу.</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>roof_aluminum_pressure_rail_m</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -4806,6 +5223,16 @@
         <v>95</v>
       </c>
       <c r="F128" s="32" t="n"/>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>price_code проставлен автоматически по точному совпадению номенклатуры; проверьте цену/единицу.</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>roof_aluminum_edge_rail_m</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -4827,6 +5254,16 @@
         <v>1146.91</v>
       </c>
       <c r="F129" s="32" t="n"/>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>price_code проставлен автоматически по точному совпадению номенклатуры; проверьте цену/единицу.</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>roof_pvc_membrane_logicroof_vrp_1_5mm_gray_roll</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -4874,6 +5311,11 @@
         <v>6001.23</v>
       </c>
       <c r="F131" s="32" t="n"/>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>Позиция кровельного прайса. price_code не проставлен автоматически, если текущие калькуляторы пока не используют эту строку напрямую.</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -4895,1478 +5337,1628 @@
         <v>2060</v>
       </c>
       <c r="F132" s="32" t="n"/>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>Позиция кровельного прайса. price_code не проставлен автоматически, если текущие калькуляторы пока не используют эту строку напрямую.</t>
+        </is>
+      </c>
     </row>
     <row r="133">
-      <c r="E133" s="29" t="n"/>
-      <c r="F133" s="32" t="n"/>
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Земляные работы</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Вынос осей фундамента, котлована на участок</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>смена</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>15000</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>axis_marking_shift</t>
+        </is>
+      </c>
     </row>
     <row r="134">
-      <c r="E134" s="29" t="n"/>
-      <c r="F134" s="32" t="n"/>
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Ж/Б монолитная плита перекрытия 1-го этажа</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Бетонирование балки бетоном марки В22,5 (М300)</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>м3</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>20000.000000</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>beam_concrete_placing_work_m3</t>
+        </is>
+      </c>
     </row>
     <row r="135">
-      <c r="E135" s="29" t="n"/>
-      <c r="F135" s="32" t="n"/>
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Гидроизоляция фундаментной плиты</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Гидроизоляция фундаментной плиты битумной мастикой в 2 слоя</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>м2</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>350</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>bitumen_waterproofing_work_m2</t>
+        </is>
+      </c>
     </row>
     <row r="136">
-      <c r="E136" s="29" t="n"/>
-      <c r="F136" s="32" t="n"/>
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Несущие стены и перемычки</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Доставка блоков, смеси</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>маш</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>28000</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>block_delivery_truck</t>
+        </is>
+      </c>
     </row>
     <row r="137">
-      <c r="E137" s="29" t="n"/>
-      <c r="F137" s="32" t="n"/>
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Несущие стены и перемычки</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Разгрузка блоков, смеси манипулятором</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>маш</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>15000</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>block_unloading_manipulator_truck</t>
+        </is>
+      </c>
     </row>
     <row r="138">
-      <c r="E138" s="29" t="n"/>
-      <c r="F138" s="32" t="n"/>
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Земляные работы</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Закладка технологических входов коммуникаций до границы дома</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>мп</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>350</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>communications_installation_m</t>
+        </is>
+      </c>
     </row>
     <row r="139">
-      <c r="E139" s="29" t="n"/>
-      <c r="F139" s="32" t="n"/>
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Земляные работы</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Материалы для устройства входов коммуникаций</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>мп</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>650</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>communications_material_m</t>
+        </is>
+      </c>
     </row>
     <row r="140">
-      <c r="E140" s="29" t="n"/>
-      <c r="F140" s="32" t="n"/>
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Ж/Б монолитная плита перекрытия 1-го этажа</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Бетон марки В22,5 (М300)</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>м3</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>6400.000000</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: requires_decision. Добавлено из калькулятора MVP, требуется проверка Елены Требуется решение по смыслу/единице перед production-использованием.</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>concrete_b22_5_m3</t>
+        </is>
+      </c>
     </row>
     <row r="141">
-      <c r="E141" s="29" t="n"/>
-      <c r="F141" s="32" t="n"/>
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Ж/Б монолитная плита перекрытия 1-го этажа</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Доставка бетона до объекта</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>рейс</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>7500.000000</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: requires_decision. Добавлено из калькулятора MVP, требуется проверка Елены Требуется решение по смыслу/единице перед production-использованием.</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>concrete_delivery_trip</t>
+        </is>
+      </c>
     </row>
     <row r="142">
-      <c r="E142" s="29" t="n"/>
-      <c r="F142" s="32" t="n"/>
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Ж/Б монолитная плита перекрытия 1-го этажа</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Бетонирование монолитной плиты перекрытия бетоном марки В22,5 (М300)</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>м3</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>12000.000000</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>concrete_placing_work_m3</t>
+        </is>
+      </c>
     </row>
     <row r="143">
-      <c r="E143" s="29" t="n"/>
-      <c r="F143" s="32" t="n"/>
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Ж/Б монолитная плита перекрытия 1-го этажа</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Работа бетононасоса 32м + гаситель</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>смена</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>38000.000000</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>concrete_pump_32m_shift</t>
+        </is>
+      </c>
     </row>
     <row r="144">
-      <c r="E144" s="29" t="n"/>
-      <c r="F144" s="32" t="n"/>
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Ж/Б монолитная плита перекрытия 1-го этажа</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Подача опалубки, арматуры автокраном</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>смена</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>30000.000000</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>crane_shift</t>
+        </is>
+      </c>
     </row>
     <row r="145">
-      <c r="E145" s="29" t="n"/>
-      <c r="F145" s="32" t="n"/>
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Несущие стены и перемычки</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Гидроизоляция поверхности под первый ряд блоков</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>м2</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>cutoff_waterproofing_under_blocks_m2</t>
+        </is>
+      </c>
     </row>
     <row r="146">
-      <c r="E146" s="29" t="n"/>
-      <c r="F146" s="32" t="n"/>
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Ж/Б монолитная плита перекрытия 1-го этажа</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Устройство утепления по наружной стороне торцов плиты, балок</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>мп</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>450.000000</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>edge_insulation_work_m</t>
+        </is>
+      </c>
     </row>
     <row r="147">
-      <c r="E147" s="29" t="n"/>
-      <c r="F147" s="32" t="n"/>
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Ж/Б монолитная плита перекрытия 1-го этажа</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Устройство утепления низа плиты</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>м2</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>900.000000</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>eps_bottom_slab_insulation_work_m2</t>
+        </is>
+      </c>
     </row>
     <row r="148">
-      <c r="E148" s="29" t="n"/>
-      <c r="F148" s="32" t="n"/>
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Устройство фундаментной плиты</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Укладка ЭППС 50мм под плитой</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>м2</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>250</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>eps_laying_work_m2</t>
+        </is>
+      </c>
     </row>
     <row r="149">
-      <c r="E149" s="29" t="n"/>
-      <c r="F149" s="32" t="n"/>
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Ж/Б монолитная плита перекрытия 1-го этажа</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Экструдированный пенополистирол Пеноплэкс Основа 100х585х1185 мм</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>м3</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>9020.000000</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>eps_penoplex_osnova_100_m3</t>
+        </is>
+      </c>
     </row>
     <row r="150">
-      <c r="E150" s="29" t="n"/>
-      <c r="F150" s="32" t="n"/>
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Гидроизоляция фундаментной плиты</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Утепление стен плиты ЭППС 100 мм</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>м2</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>eps_wall_insulation_work_m2</t>
+        </is>
+      </c>
     </row>
     <row r="151">
-      <c r="E151" s="29" t="n"/>
-      <c r="F151" s="32" t="n"/>
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Земляные работы</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Механизированная разработка грунта, Экскаватор JCB</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>смена</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>22000</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>excavator_jcb_shift</t>
+        </is>
+      </c>
     </row>
     <row r="152">
-      <c r="E152" s="29" t="n"/>
-      <c r="F152" s="32" t="n"/>
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Ж/Б монолитная плита перекрытия 1-го этажа</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Расходные материалы для установки опалубки (смазка; звездочки ПВХ, трубки)</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>9759.080000</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>formwork_consumables_m2</t>
+        </is>
+      </c>
     </row>
     <row r="153">
-      <c r="E153" s="29" t="n"/>
-      <c r="F153" s="32" t="n"/>
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Ж/Б монолитная плита перекрытия 1-го этажа</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Доставка, вывоз опалубки манипулятором</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>маш</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>20000.000000</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>formwork_delivery_truck</t>
+        </is>
+      </c>
     </row>
     <row r="154">
-      <c r="E154" s="29" t="n"/>
-      <c r="F154" s="32" t="n"/>
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Устройство фундаментной плиты</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Демонтаж опалубки после завершения бетонирования</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>м2</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>formwork_dismantling_work_m2</t>
+        </is>
+      </c>
     </row>
     <row r="155">
-      <c r="E155" s="29" t="n"/>
-      <c r="F155" s="32" t="n"/>
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Ж/Б монолитная плита перекрытия 1-го этажа</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Комплект опалубки (телескопические стойки, унивилки, треноги, водостойкая фанера, поперечные и продольные балки двутавровые)</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>м2</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>600.000000</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>formwork_rental_m2</t>
+        </is>
+      </c>
     </row>
     <row r="156">
-      <c r="E156" s="29" t="n"/>
-      <c r="F156" s="32" t="n"/>
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Несущие стены и перемычки</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Обкладка дымохода и вентканалов 150 мм</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>м2</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>1200</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>gas_block_cladding_work_m2</t>
+        </is>
+      </c>
     </row>
     <row r="157">
-      <c r="E157" s="29" t="n"/>
-      <c r="F157" s="32" t="n"/>
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Несущие стены и перемычки</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Газобетонный блок D400 600x400x250 мм</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>м3</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>6000</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>gas_block_d400_m3</t>
+        </is>
+      </c>
     </row>
     <row r="158">
-      <c r="E158" s="29" t="n"/>
-      <c r="F158" s="32" t="n"/>
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Несущие стены и перемычки</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Газобетонный блок D500 600x150x250 мм</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>м3</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>5600</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>gas_block_d500_150_m3</t>
+        </is>
+      </c>
     </row>
     <row r="159">
-      <c r="E159" s="29" t="n"/>
-      <c r="F159" s="32" t="n"/>
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Несущие стены и перемычки</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Газобетонный блок D500 600x250x250 мм</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>м3</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>5500</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>gas_block_d500_m3</t>
+        </is>
+      </c>
     </row>
     <row r="160">
-      <c r="E160" s="29" t="n"/>
-      <c r="F160" s="32" t="n"/>
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Несущие стены и перемычки</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Кладка внешних, внутренних стен из газобетонных блоков</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>м3</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>7000</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>gas_block_masonry_work_m3</t>
+        </is>
+      </c>
     </row>
     <row r="161">
-      <c r="E161" s="29" t="n"/>
-      <c r="F161" s="32" t="n"/>
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Земляные работы</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Укладка геотекстиля</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>м2</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>geotextile_laying_m2</t>
+        </is>
+      </c>
     </row>
     <row r="162">
-      <c r="E162" s="29" t="n"/>
-      <c r="F162" s="32" t="n"/>
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Несущие стены и перемычки</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Бетонирование перемычек</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>мп</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>lintel_concreting_work_m</t>
+        </is>
+      </c>
     </row>
     <row r="163">
-      <c r="E163" s="29" t="n"/>
-      <c r="F163" s="32" t="n"/>
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Несущие стены и перемычки</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Перенос, подъём бетона вручную</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>м3</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>5000</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>manual_concrete_lifting_m3</t>
+        </is>
+      </c>
     </row>
     <row r="164">
-      <c r="E164" s="29" t="n"/>
-      <c r="F164" s="32" t="n"/>
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Земляные работы</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Доработка грунта вручную</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>м3</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>1200</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>manual_excavation_m3</t>
+        </is>
+      </c>
     </row>
     <row r="165">
-      <c r="E165" s="29" t="n"/>
-      <c r="F165" s="32" t="n"/>
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Ж/Б монолитная плита перекрытия 1-го этажа</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Доставка арматуры, металла</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>маш</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>22000.000000</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>metal_delivery_truck</t>
+        </is>
+      </c>
     </row>
     <row r="166">
-      <c r="E166" s="29" t="n"/>
-      <c r="F166" s="32" t="n"/>
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Устройство фундаментной плиты</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Монтаж мембраны PLANTER стандарт</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>м2</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>planter_membrane_installation_work_m2</t>
+        </is>
+      </c>
     </row>
     <row r="167">
-      <c r="E167" s="29" t="n"/>
-      <c r="F167" s="32" t="n"/>
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>КРОВЕЛЬНОЕ ПОКРЫТИЕ ДОМА</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Подъем материалов автокраном</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>смена</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>30000</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>roof_crane_lifting_shift</t>
+        </is>
+      </c>
     </row>
     <row r="168">
-      <c r="E168" s="29" t="n"/>
-      <c r="F168" s="32" t="n"/>
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>КРОВЕЛЬНОЕ ПОКРЫТИЕ ДОМА</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Геотекстиль ТЕХНОНИКОЛЬ ПРОФ Кровля 300, 2х50м</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>м2</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>111.76</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: requires_decision. Добавлено из калькулятора MVP, требуется проверка Елены Требуется решение по смыслу/единице перед production-использованием.</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>roof_geotextile_technonikol_prof_300_m2</t>
+        </is>
+      </c>
     </row>
     <row r="169">
-      <c r="E169" s="29" t="n"/>
-      <c r="F169" s="32" t="n"/>
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>КРОВЕЛЬНОЕ ПОКРЫТИЕ ДОМА</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Устройство внутреннего водостока (ПВХ Ф110мм) (ориентировочно)</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>мп</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>2500</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>roof_internal_drain_pvc_110mm_m</t>
+        </is>
+      </c>
     </row>
     <row r="170">
-      <c r="E170" s="29" t="n"/>
-      <c r="F170" s="32" t="n"/>
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>КРОВЕЛЬНОЕ ПОКРЫТИЕ ДОМА</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Установка воронки кровельной (с обжимным мет. фланцем с обогревом 110х450мм) (без пробивки отверстий)</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>5000</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>roof_internal_drain_with_heating_item</t>
+        </is>
+      </c>
     </row>
     <row r="171">
-      <c r="E171" s="29" t="n"/>
-      <c r="F171" s="32" t="n"/>
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>КРОВЕЛЬНОЕ ПОКРЫТИЕ ДОМА</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Установка воронки парапетной (без пробивки отверстий)</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>5000</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>roof_parapet_drain_item</t>
+        </is>
+      </c>
     </row>
     <row r="172">
-      <c r="E172" s="29" t="n"/>
-      <c r="F172" s="32" t="n"/>
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Несущие стены и перемычки</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Пескобетон М300 40 кг</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>375</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>sand_concrete_bag</t>
+        </is>
+      </c>
     </row>
     <row r="173">
-      <c r="E173" s="29" t="n"/>
-      <c r="F173" s="32" t="n"/>
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Земляные работы</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Отсыпка дна котлована, засыпка под плитой песком с трамбованием</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>м3</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>1200</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>sand_filling_work_m3</t>
+        </is>
+      </c>
     </row>
     <row r="174">
-      <c r="E174" s="29" t="n"/>
-      <c r="F174" s="32" t="n"/>
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Земляные работы</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Песок строительный</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>м3</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>sand_m3</t>
+        </is>
+      </c>
     </row>
     <row r="175">
-      <c r="E175" s="29" t="n"/>
-      <c r="F175" s="32" t="n"/>
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Земляные работы</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Перемещение песка вручную</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>м3</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>sand_manual_moving_m3</t>
+        </is>
+      </c>
     </row>
     <row r="176">
-      <c r="E176" s="29" t="n"/>
-      <c r="F176" s="32" t="n"/>
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Несущие стены и перемычки</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Устройство лесов, подмостей для кладки, демонтаж лесов</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>компл</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>20000</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>scaffolding_setup_dismantling_work_set</t>
+        </is>
+      </c>
     </row>
     <row r="177">
-      <c r="E177" s="29" t="n"/>
-      <c r="F177" s="32" t="n"/>
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>ВЕНТИЛЯЦИОННЫЕ КАНАЛЫ Schiedel</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Доставка вентканалов</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>маш</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>15000</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>schiedel_delivery_truck</t>
+        </is>
+      </c>
     </row>
     <row r="178">
-      <c r="E178" s="29" t="n"/>
-      <c r="F178" s="32" t="n"/>
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Ж/Б монолитная плита перекрытия 1-го этажа</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Технический надзор</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>5000.000000</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>technical_supervision_fixed</t>
+        </is>
+      </c>
     </row>
     <row r="179">
-      <c r="E179" s="29" t="n"/>
-      <c r="F179" s="32" t="n"/>
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Устройство фундаментной плиты</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Устройство и монтаж термовкладыша 150*400*250мм шаг 200мм</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>мп</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>thermal_insert_installation_work_m</t>
+        </is>
+      </c>
     </row>
     <row r="180">
-      <c r="E180" s="29" t="n"/>
-      <c r="F180" s="32" t="n"/>
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Устройство фундаментной плиты</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Монтаж опалубки из пиломатериалов для отбортовки плиты</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>м2</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>timber_formwork_installation_work_m2</t>
+        </is>
+      </c>
     </row>
     <row r="181">
-      <c r="E181" s="29" t="n"/>
-      <c r="F181" s="32" t="n"/>
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Ж/Б монолитная плита перекрытия 1-го этажа</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Пиломатериал обрезной для устройства опалубки ГОСТ</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>м3</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>21499.997319</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>timber_m3</t>
+        </is>
+      </c>
     </row>
     <row r="182">
-      <c r="E182" s="29" t="n"/>
-      <c r="F182" s="32" t="n"/>
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Несущие стены и перемычки</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Резка блока под перемычку (U-блок)</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>u_block_lintel_cutting_item</t>
+        </is>
+      </c>
     </row>
     <row r="183">
-      <c r="E183" s="29" t="n"/>
-      <c r="F183" s="32" t="n"/>
-    </row>
-    <row r="184">
-      <c r="E184" s="29" t="n"/>
-      <c r="F184" s="32" t="n"/>
-    </row>
-    <row r="185">
-      <c r="E185" s="29" t="n"/>
-      <c r="F185" s="32" t="n"/>
-    </row>
-    <row r="186">
-      <c r="E186" s="29" t="n"/>
-      <c r="F186" s="32" t="n"/>
-    </row>
-    <row r="187">
-      <c r="E187" s="29" t="n"/>
-      <c r="F187" s="32" t="n"/>
-    </row>
-    <row r="188">
-      <c r="E188" s="29" t="n"/>
-      <c r="F188" s="32" t="n"/>
-    </row>
-    <row r="189">
-      <c r="E189" s="29" t="n"/>
-      <c r="F189" s="32" t="n"/>
-    </row>
-    <row r="190">
-      <c r="E190" s="29" t="n"/>
-      <c r="F190" s="32" t="n"/>
-    </row>
-    <row r="191">
-      <c r="E191" s="29" t="n"/>
-      <c r="F191" s="32" t="n"/>
-    </row>
-    <row r="192">
-      <c r="E192" s="29" t="n"/>
-      <c r="F192" s="32" t="n"/>
-    </row>
-    <row r="193">
-      <c r="E193" s="29" t="n"/>
-      <c r="F193" s="32" t="n"/>
-    </row>
-    <row r="194">
-      <c r="E194" s="29" t="n"/>
-      <c r="F194" s="32" t="n"/>
-    </row>
-    <row r="195">
-      <c r="E195" s="29" t="n"/>
-      <c r="F195" s="32" t="n"/>
-    </row>
-    <row r="196">
-      <c r="E196" s="29" t="n"/>
-      <c r="F196" s="32" t="n"/>
-    </row>
-    <row r="197">
-      <c r="E197" s="29" t="n"/>
-      <c r="F197" s="32" t="n"/>
-    </row>
-    <row r="198">
-      <c r="E198" s="29" t="n"/>
-      <c r="F198" s="32" t="n"/>
-    </row>
-    <row r="199">
-      <c r="E199" s="29" t="n"/>
-      <c r="F199" s="32" t="n"/>
-    </row>
-    <row r="200">
-      <c r="E200" s="29" t="n"/>
-      <c r="F200" s="32" t="n"/>
-    </row>
-    <row r="201">
-      <c r="E201" s="29" t="n"/>
-      <c r="F201" s="32" t="n"/>
-    </row>
-    <row r="202">
-      <c r="E202" s="29" t="n"/>
-      <c r="F202" s="32" t="n"/>
-    </row>
-    <row r="203">
-      <c r="E203" s="29" t="n"/>
-      <c r="F203" s="32" t="n"/>
-    </row>
-    <row r="204">
-      <c r="E204" s="29" t="n"/>
-      <c r="F204" s="32" t="n"/>
-    </row>
-    <row r="205">
-      <c r="E205" s="29" t="n"/>
-      <c r="F205" s="32" t="n"/>
-    </row>
-    <row r="206">
-      <c r="E206" s="29" t="n"/>
-      <c r="F206" s="32" t="n"/>
-    </row>
-    <row r="207">
-      <c r="E207" s="29" t="n"/>
-      <c r="F207" s="32" t="n"/>
-    </row>
-    <row r="208">
-      <c r="E208" s="29" t="n"/>
-      <c r="F208" s="32" t="n"/>
-    </row>
-    <row r="209">
-      <c r="E209" s="29" t="n"/>
-      <c r="F209" s="32" t="n"/>
-    </row>
-    <row r="210">
-      <c r="E210" s="29" t="n"/>
-      <c r="F210" s="32" t="n"/>
-    </row>
-    <row r="211">
-      <c r="E211" s="29" t="n"/>
-      <c r="F211" s="32" t="n"/>
-    </row>
-    <row r="212">
-      <c r="E212" s="29" t="n"/>
-      <c r="F212" s="32" t="n"/>
-    </row>
-    <row r="213">
-      <c r="E213" s="29" t="n"/>
-      <c r="F213" s="32" t="n"/>
-    </row>
-    <row r="214">
-      <c r="E214" s="29" t="n"/>
-      <c r="F214" s="32" t="n"/>
-    </row>
-    <row r="215">
-      <c r="E215" s="29" t="n"/>
-      <c r="F215" s="32" t="n"/>
-    </row>
-    <row r="216">
-      <c r="E216" s="29" t="n"/>
-      <c r="F216" s="32" t="n"/>
-    </row>
-    <row r="217">
-      <c r="E217" s="29" t="n"/>
-      <c r="F217" s="32" t="n"/>
-    </row>
-    <row r="218">
-      <c r="E218" s="29" t="n"/>
-      <c r="F218" s="32" t="n"/>
-    </row>
-    <row r="219">
-      <c r="E219" s="29" t="n"/>
-      <c r="F219" s="32" t="n"/>
-    </row>
-    <row r="220">
-      <c r="E220" s="29" t="n"/>
-      <c r="F220" s="32" t="n"/>
-    </row>
-    <row r="221">
-      <c r="E221" s="29" t="n"/>
-      <c r="F221" s="32" t="n"/>
-    </row>
-    <row r="222">
-      <c r="E222" s="29" t="n"/>
-      <c r="F222" s="32" t="n"/>
-    </row>
-    <row r="223">
-      <c r="E223" s="29" t="n"/>
-      <c r="F223" s="32" t="n"/>
-    </row>
-    <row r="224">
-      <c r="E224" s="29" t="n"/>
-      <c r="F224" s="32" t="n"/>
-    </row>
-    <row r="225">
-      <c r="E225" s="29" t="n"/>
-      <c r="F225" s="32" t="n"/>
-    </row>
-    <row r="226">
-      <c r="E226" s="29" t="n"/>
-      <c r="F226" s="32" t="n"/>
-    </row>
-    <row r="227">
-      <c r="E227" s="29" t="n"/>
-      <c r="F227" s="32" t="n"/>
-    </row>
-    <row r="228">
-      <c r="E228" s="29" t="n"/>
-      <c r="F228" s="32" t="n"/>
-    </row>
-    <row r="229">
-      <c r="E229" s="29" t="n"/>
-      <c r="F229" s="32" t="n"/>
-    </row>
-    <row r="230">
-      <c r="E230" s="29" t="n"/>
-      <c r="F230" s="32" t="n"/>
-    </row>
-    <row r="231">
-      <c r="E231" s="29" t="n"/>
-      <c r="F231" s="32" t="n"/>
-    </row>
-    <row r="232">
-      <c r="E232" s="29" t="n"/>
-      <c r="F232" s="32" t="n"/>
-    </row>
-    <row r="233">
-      <c r="E233" s="29" t="n"/>
-      <c r="F233" s="32" t="n"/>
-    </row>
-    <row r="234">
-      <c r="E234" s="29" t="n"/>
-      <c r="F234" s="32" t="n"/>
-    </row>
-    <row r="235">
-      <c r="E235" s="29" t="n"/>
-      <c r="F235" s="32" t="n"/>
-    </row>
-    <row r="236">
-      <c r="E236" s="29" t="n"/>
-      <c r="F236" s="32" t="n"/>
-    </row>
-    <row r="237">
-      <c r="E237" s="29" t="n"/>
-      <c r="F237" s="32" t="n"/>
-    </row>
-    <row r="238">
-      <c r="E238" s="29" t="n"/>
-      <c r="F238" s="32" t="n"/>
-    </row>
-    <row r="239">
-      <c r="E239" s="29" t="n"/>
-      <c r="F239" s="32" t="n"/>
-    </row>
-    <row r="240">
-      <c r="E240" s="29" t="n"/>
-      <c r="F240" s="32" t="n"/>
-    </row>
-    <row r="241">
-      <c r="E241" s="29" t="n"/>
-      <c r="F241" s="32" t="n"/>
-    </row>
-    <row r="242">
-      <c r="E242" s="29" t="n"/>
-      <c r="F242" s="32" t="n"/>
-    </row>
-    <row r="243">
-      <c r="E243" s="29" t="n"/>
-      <c r="F243" s="32" t="n"/>
-    </row>
-    <row r="244">
-      <c r="E244" s="29" t="n"/>
-      <c r="F244" s="32" t="n"/>
-    </row>
-    <row r="245">
-      <c r="E245" s="29" t="n"/>
-      <c r="F245" s="32" t="n"/>
-    </row>
-    <row r="246">
-      <c r="E246" s="29" t="n"/>
-      <c r="F246" s="32" t="n"/>
-    </row>
-    <row r="247">
-      <c r="E247" s="29" t="n"/>
-      <c r="F247" s="32" t="n"/>
-    </row>
-    <row r="248">
-      <c r="E248" s="29" t="n"/>
-      <c r="F248" s="32" t="n"/>
-    </row>
-    <row r="249">
-      <c r="E249" s="29" t="n"/>
-      <c r="F249" s="32" t="n"/>
-    </row>
-    <row r="250">
-      <c r="E250" s="29" t="n"/>
-      <c r="F250" s="32" t="n"/>
-    </row>
-    <row r="251">
-      <c r="E251" s="29" t="n"/>
-      <c r="F251" s="32" t="n"/>
-    </row>
-    <row r="252">
-      <c r="E252" s="29" t="n"/>
-      <c r="F252" s="32" t="n"/>
-    </row>
-    <row r="253">
-      <c r="E253" s="29" t="n"/>
-      <c r="F253" s="32" t="n"/>
-    </row>
-    <row r="254">
-      <c r="E254" s="29" t="n"/>
-      <c r="F254" s="32" t="n"/>
-    </row>
-    <row r="255">
-      <c r="E255" s="29" t="n"/>
-      <c r="F255" s="32" t="n"/>
-    </row>
-    <row r="256">
-      <c r="E256" s="29" t="n"/>
-      <c r="F256" s="32" t="n"/>
-    </row>
-    <row r="257">
-      <c r="E257" s="29" t="n"/>
-      <c r="F257" s="32" t="n"/>
-    </row>
-    <row r="258">
-      <c r="E258" s="29" t="n"/>
-      <c r="F258" s="32" t="n"/>
-    </row>
-    <row r="259">
-      <c r="E259" s="29" t="n"/>
-      <c r="F259" s="32" t="n"/>
-    </row>
-    <row r="260">
-      <c r="E260" s="29" t="n"/>
-      <c r="F260" s="32" t="n"/>
-    </row>
-    <row r="261">
-      <c r="E261" s="29" t="n"/>
-      <c r="F261" s="32" t="n"/>
-    </row>
-    <row r="262">
-      <c r="E262" s="29" t="n"/>
-      <c r="F262" s="32" t="n"/>
-    </row>
-    <row r="263">
-      <c r="E263" s="29" t="n"/>
-      <c r="F263" s="32" t="n"/>
-    </row>
-    <row r="264">
-      <c r="E264" s="29" t="n"/>
-      <c r="F264" s="32" t="n"/>
-    </row>
-    <row r="265">
-      <c r="E265" s="29" t="n"/>
-      <c r="F265" s="32" t="n"/>
-    </row>
-    <row r="266">
-      <c r="E266" s="29" t="n"/>
-      <c r="F266" s="32" t="n"/>
-    </row>
-    <row r="267">
-      <c r="E267" s="29" t="n"/>
-      <c r="F267" s="32" t="n"/>
-    </row>
-    <row r="268">
-      <c r="E268" s="29" t="n"/>
-      <c r="F268" s="32" t="n"/>
-    </row>
-    <row r="269">
-      <c r="E269" s="29" t="n"/>
-      <c r="F269" s="32" t="n"/>
-    </row>
-    <row r="270">
-      <c r="E270" s="29" t="n"/>
-      <c r="F270" s="32" t="n"/>
-    </row>
-    <row r="271">
-      <c r="E271" s="29" t="n"/>
-      <c r="F271" s="32" t="n"/>
-    </row>
-    <row r="272">
-      <c r="E272" s="29" t="n"/>
-      <c r="F272" s="32" t="n"/>
-    </row>
-    <row r="273">
-      <c r="E273" s="29" t="n"/>
-      <c r="F273" s="32" t="n"/>
-    </row>
-    <row r="274">
-      <c r="E274" s="29" t="n"/>
-      <c r="F274" s="32" t="n"/>
-    </row>
-    <row r="275">
-      <c r="E275" s="29" t="n"/>
-      <c r="F275" s="32" t="n"/>
-    </row>
-    <row r="276">
-      <c r="E276" s="29" t="n"/>
-      <c r="F276" s="32" t="n"/>
-    </row>
-    <row r="277">
-      <c r="E277" s="29" t="n"/>
-      <c r="F277" s="32" t="n"/>
-    </row>
-    <row r="278">
-      <c r="E278" s="29" t="n"/>
-      <c r="F278" s="32" t="n"/>
-    </row>
-    <row r="279">
-      <c r="E279" s="29" t="n"/>
-      <c r="F279" s="32" t="n"/>
-    </row>
-    <row r="280">
-      <c r="E280" s="29" t="n"/>
-      <c r="F280" s="32" t="n"/>
-    </row>
-    <row r="281">
-      <c r="E281" s="29" t="n"/>
-      <c r="F281" s="32" t="n"/>
-    </row>
-    <row r="282">
-      <c r="E282" s="29" t="n"/>
-      <c r="F282" s="32" t="n"/>
-    </row>
-    <row r="283">
-      <c r="E283" s="29" t="n"/>
-      <c r="F283" s="32" t="n"/>
-    </row>
-    <row r="284">
-      <c r="E284" s="29" t="n"/>
-      <c r="F284" s="32" t="n"/>
-    </row>
-    <row r="285">
-      <c r="E285" s="29" t="n"/>
-      <c r="F285" s="32" t="n"/>
-    </row>
-    <row r="286">
-      <c r="E286" s="29" t="n"/>
-      <c r="F286" s="32" t="n"/>
-    </row>
-    <row r="287">
-      <c r="E287" s="29" t="n"/>
-      <c r="F287" s="32" t="n"/>
-    </row>
-    <row r="288">
-      <c r="E288" s="29" t="n"/>
-      <c r="F288" s="32" t="n"/>
-    </row>
-    <row r="289">
-      <c r="E289" s="29" t="n"/>
-      <c r="F289" s="32" t="n"/>
-    </row>
-    <row r="290">
-      <c r="E290" s="29" t="n"/>
-      <c r="F290" s="32" t="n"/>
-    </row>
-    <row r="291">
-      <c r="E291" s="29" t="n"/>
-      <c r="F291" s="32" t="n"/>
-    </row>
-    <row r="292">
-      <c r="E292" s="29" t="n"/>
-      <c r="F292" s="32" t="n"/>
-    </row>
-    <row r="293">
-      <c r="E293" s="29" t="n"/>
-      <c r="F293" s="32" t="n"/>
-    </row>
-    <row r="294">
-      <c r="E294" s="29" t="n"/>
-      <c r="F294" s="32" t="n"/>
-    </row>
-    <row r="295">
-      <c r="E295" s="29" t="n"/>
-      <c r="F295" s="32" t="n"/>
-    </row>
-    <row r="296">
-      <c r="E296" s="29" t="n"/>
-      <c r="F296" s="32" t="n"/>
-    </row>
-    <row r="297">
-      <c r="E297" s="29" t="n"/>
-      <c r="F297" s="32" t="n"/>
-    </row>
-    <row r="298">
-      <c r="E298" s="29" t="n"/>
-      <c r="F298" s="32" t="n"/>
-    </row>
-    <row r="299">
-      <c r="E299" s="29" t="n"/>
-      <c r="F299" s="32" t="n"/>
-    </row>
-    <row r="300">
-      <c r="E300" s="29" t="n"/>
-      <c r="F300" s="32" t="n"/>
-    </row>
-    <row r="301">
-      <c r="E301" s="29" t="n"/>
-      <c r="F301" s="32" t="n"/>
-    </row>
-    <row r="302">
-      <c r="E302" s="29" t="n"/>
-      <c r="F302" s="32" t="n"/>
-    </row>
-    <row r="303">
-      <c r="E303" s="29" t="n"/>
-      <c r="F303" s="32" t="n"/>
-    </row>
-    <row r="304">
-      <c r="E304" s="29" t="n"/>
-      <c r="F304" s="32" t="n"/>
-    </row>
-    <row r="305">
-      <c r="E305" s="29" t="n"/>
-      <c r="F305" s="32" t="n"/>
-    </row>
-    <row r="306">
-      <c r="E306" s="29" t="n"/>
-      <c r="F306" s="32" t="n"/>
-    </row>
-    <row r="307">
-      <c r="E307" s="29" t="n"/>
-      <c r="F307" s="32" t="n"/>
-    </row>
-    <row r="308">
-      <c r="E308" s="29" t="n"/>
-      <c r="F308" s="32" t="n"/>
-    </row>
-    <row r="309">
-      <c r="E309" s="29" t="n"/>
-      <c r="F309" s="32" t="n"/>
-    </row>
-    <row r="310">
-      <c r="E310" s="29" t="n"/>
-      <c r="F310" s="32" t="n"/>
-    </row>
-    <row r="311">
-      <c r="E311" s="29" t="n"/>
-      <c r="F311" s="32" t="n"/>
-    </row>
-    <row r="312">
-      <c r="E312" s="29" t="n"/>
-      <c r="F312" s="32" t="n"/>
-    </row>
-    <row r="313">
-      <c r="E313" s="29" t="n"/>
-      <c r="F313" s="32" t="n"/>
-    </row>
-    <row r="314">
-      <c r="E314" s="29" t="n"/>
-      <c r="F314" s="32" t="n"/>
-    </row>
-    <row r="315">
-      <c r="E315" s="29" t="n"/>
-      <c r="F315" s="32" t="n"/>
-    </row>
-    <row r="316">
-      <c r="E316" s="29" t="n"/>
-      <c r="F316" s="32" t="n"/>
-    </row>
-    <row r="317">
-      <c r="E317" s="29" t="n"/>
-      <c r="F317" s="32" t="n"/>
-    </row>
-    <row r="318">
-      <c r="E318" s="29" t="n"/>
-      <c r="F318" s="32" t="n"/>
-    </row>
-    <row r="319">
-      <c r="E319" s="29" t="n"/>
-      <c r="F319" s="32" t="n"/>
-    </row>
-    <row r="320">
-      <c r="E320" s="29" t="n"/>
-      <c r="F320" s="32" t="n"/>
-    </row>
-    <row r="321">
-      <c r="E321" s="29" t="n"/>
-      <c r="F321" s="32" t="n"/>
-    </row>
-    <row r="322">
-      <c r="E322" s="29" t="n"/>
-      <c r="F322" s="32" t="n"/>
-    </row>
-    <row r="323">
-      <c r="E323" s="29" t="n"/>
-      <c r="F323" s="32" t="n"/>
-    </row>
-    <row r="324">
-      <c r="E324" s="29" t="n"/>
-      <c r="F324" s="32" t="n"/>
-    </row>
-    <row r="325">
-      <c r="E325" s="29" t="n"/>
-      <c r="F325" s="32" t="n"/>
-    </row>
-    <row r="326">
-      <c r="E326" s="29" t="n"/>
-      <c r="F326" s="32" t="n"/>
-    </row>
-    <row r="327">
-      <c r="E327" s="29" t="n"/>
-      <c r="F327" s="32" t="n"/>
-    </row>
-    <row r="328">
-      <c r="E328" s="29" t="n"/>
-      <c r="F328" s="32" t="n"/>
-    </row>
-    <row r="329">
-      <c r="E329" s="29" t="n"/>
-      <c r="F329" s="32" t="n"/>
-    </row>
-    <row r="330">
-      <c r="E330" s="29" t="n"/>
-      <c r="F330" s="32" t="n"/>
-    </row>
-    <row r="331">
-      <c r="E331" s="29" t="n"/>
-      <c r="F331" s="32" t="n"/>
-    </row>
-    <row r="332">
-      <c r="E332" s="29" t="n"/>
-      <c r="F332" s="32" t="n"/>
-    </row>
-    <row r="333">
-      <c r="E333" s="29" t="n"/>
-      <c r="F333" s="32" t="n"/>
-    </row>
-    <row r="334">
-      <c r="E334" s="29" t="n"/>
-      <c r="F334" s="32" t="n"/>
-    </row>
-    <row r="335">
-      <c r="E335" s="29" t="n"/>
-      <c r="F335" s="32" t="n"/>
-    </row>
-    <row r="336">
-      <c r="E336" s="29" t="n"/>
-      <c r="F336" s="32" t="n"/>
-    </row>
-    <row r="337">
-      <c r="E337" s="29" t="n"/>
-      <c r="F337" s="32" t="n"/>
-    </row>
-    <row r="338">
-      <c r="E338" s="29" t="n"/>
-      <c r="F338" s="32" t="n"/>
-    </row>
-    <row r="339">
-      <c r="E339" s="29" t="n"/>
-      <c r="F339" s="32" t="n"/>
-    </row>
-    <row r="340">
-      <c r="E340" s="29" t="n"/>
-      <c r="F340" s="32" t="n"/>
-    </row>
-    <row r="341">
-      <c r="E341" s="29" t="n"/>
-      <c r="F341" s="32" t="n"/>
-    </row>
-    <row r="342">
-      <c r="E342" s="29" t="n"/>
-      <c r="F342" s="32" t="n"/>
-    </row>
-    <row r="343">
-      <c r="E343" s="29" t="n"/>
-      <c r="F343" s="32" t="n"/>
-    </row>
-    <row r="344">
-      <c r="E344" s="29" t="n"/>
-      <c r="F344" s="32" t="n"/>
-    </row>
-    <row r="345">
-      <c r="E345" s="29" t="n"/>
-      <c r="F345" s="32" t="n"/>
-    </row>
-    <row r="346">
-      <c r="E346" s="29" t="n"/>
-      <c r="F346" s="32" t="n"/>
-    </row>
-    <row r="347">
-      <c r="E347" s="29" t="n"/>
-      <c r="F347" s="32" t="n"/>
-    </row>
-    <row r="348">
-      <c r="E348" s="29" t="n"/>
-      <c r="F348" s="32" t="n"/>
-    </row>
-    <row r="349">
-      <c r="E349" s="29" t="n"/>
-      <c r="F349" s="32" t="n"/>
-    </row>
-    <row r="350">
-      <c r="E350" s="29" t="n"/>
-      <c r="F350" s="32" t="n"/>
-    </row>
-    <row r="351">
-      <c r="E351" s="29" t="n"/>
-      <c r="F351" s="32" t="n"/>
-    </row>
-    <row r="352">
-      <c r="E352" s="29" t="n"/>
-      <c r="F352" s="32" t="n"/>
-    </row>
-    <row r="353">
-      <c r="E353" s="29" t="n"/>
-      <c r="F353" s="32" t="n"/>
-    </row>
-    <row r="354">
-      <c r="E354" s="29" t="n"/>
-      <c r="F354" s="32" t="n"/>
-    </row>
-    <row r="355">
-      <c r="E355" s="29" t="n"/>
-      <c r="F355" s="32" t="n"/>
-    </row>
-    <row r="356">
-      <c r="E356" s="29" t="n"/>
-      <c r="F356" s="32" t="n"/>
-    </row>
-    <row r="357">
-      <c r="E357" s="29" t="n"/>
-      <c r="F357" s="32" t="n"/>
-    </row>
-    <row r="358">
-      <c r="E358" s="29" t="n"/>
-      <c r="F358" s="32" t="n"/>
-    </row>
-    <row r="359">
-      <c r="E359" s="29" t="n"/>
-      <c r="F359" s="32" t="n"/>
-    </row>
-    <row r="360">
-      <c r="E360" s="29" t="n"/>
-      <c r="F360" s="32" t="n"/>
-    </row>
-    <row r="361">
-      <c r="E361" s="29" t="n"/>
-      <c r="F361" s="32" t="n"/>
-    </row>
-    <row r="362">
-      <c r="E362" s="29" t="n"/>
-      <c r="F362" s="32" t="n"/>
-    </row>
-    <row r="363">
-      <c r="E363" s="29" t="n"/>
-      <c r="F363" s="32" t="n"/>
-    </row>
-    <row r="364">
-      <c r="E364" s="29" t="n"/>
-      <c r="F364" s="32" t="n"/>
-    </row>
-    <row r="365">
-      <c r="E365" s="29" t="n"/>
-      <c r="F365" s="32" t="n"/>
-    </row>
-    <row r="366">
-      <c r="E366" s="29" t="n"/>
-      <c r="F366" s="32" t="n"/>
-    </row>
-    <row r="367">
-      <c r="E367" s="29" t="n"/>
-      <c r="F367" s="32" t="n"/>
-    </row>
-    <row r="368">
-      <c r="E368" s="29" t="n"/>
-      <c r="F368" s="32" t="n"/>
-    </row>
-    <row r="369">
-      <c r="E369" s="29" t="n"/>
-      <c r="F369" s="32" t="n"/>
-    </row>
-    <row r="370">
-      <c r="E370" s="29" t="n"/>
-      <c r="F370" s="32" t="n"/>
-    </row>
-    <row r="371">
-      <c r="E371" s="29" t="n"/>
-      <c r="F371" s="32" t="n"/>
-    </row>
-    <row r="372">
-      <c r="E372" s="29" t="n"/>
-      <c r="F372" s="32" t="n"/>
-    </row>
-    <row r="373">
-      <c r="E373" s="29" t="n"/>
-      <c r="F373" s="32" t="n"/>
-    </row>
-    <row r="374">
-      <c r="E374" s="29" t="n"/>
-      <c r="F374" s="32" t="n"/>
-    </row>
-    <row r="375">
-      <c r="E375" s="29" t="n"/>
-      <c r="F375" s="32" t="n"/>
-    </row>
-    <row r="376">
-      <c r="E376" s="29" t="n"/>
-      <c r="F376" s="32" t="n"/>
-    </row>
-    <row r="377">
-      <c r="E377" s="29" t="n"/>
-      <c r="F377" s="32" t="n"/>
-    </row>
-    <row r="378">
-      <c r="E378" s="29" t="n"/>
-      <c r="F378" s="32" t="n"/>
-    </row>
-    <row r="379">
-      <c r="E379" s="29" t="n"/>
-      <c r="F379" s="32" t="n"/>
-    </row>
-    <row r="380">
-      <c r="E380" s="29" t="n"/>
-      <c r="F380" s="32" t="n"/>
-    </row>
-    <row r="381">
-      <c r="E381" s="29" t="n"/>
-      <c r="F381" s="32" t="n"/>
-    </row>
-    <row r="382">
-      <c r="E382" s="29" t="n"/>
-      <c r="F382" s="32" t="n"/>
-    </row>
-    <row r="383">
-      <c r="E383" s="29" t="n"/>
-      <c r="F383" s="32" t="n"/>
-    </row>
-    <row r="384">
-      <c r="E384" s="29" t="n"/>
-      <c r="F384" s="32" t="n"/>
-    </row>
-    <row r="385">
-      <c r="E385" s="29" t="n"/>
-      <c r="F385" s="32" t="n"/>
-    </row>
-    <row r="386">
-      <c r="E386" s="29" t="n"/>
-      <c r="F386" s="32" t="n"/>
-    </row>
-    <row r="387">
-      <c r="E387" s="29" t="n"/>
-      <c r="F387" s="32" t="n"/>
-    </row>
-    <row r="388">
-      <c r="E388" s="29" t="n"/>
-      <c r="F388" s="32" t="n"/>
-    </row>
-    <row r="389">
-      <c r="E389" s="29" t="n"/>
-      <c r="F389" s="32" t="n"/>
-    </row>
-    <row r="390">
-      <c r="E390" s="29" t="n"/>
-      <c r="F390" s="32" t="n"/>
-    </row>
-    <row r="391">
-      <c r="E391" s="29" t="n"/>
-      <c r="F391" s="32" t="n"/>
-    </row>
-    <row r="392">
-      <c r="E392" s="29" t="n"/>
-      <c r="F392" s="32" t="n"/>
-    </row>
-    <row r="393">
-      <c r="E393" s="29" t="n"/>
-      <c r="F393" s="32" t="n"/>
-    </row>
-    <row r="394">
-      <c r="E394" s="29" t="n"/>
-      <c r="F394" s="32" t="n"/>
-    </row>
-    <row r="395">
-      <c r="E395" s="29" t="n"/>
-      <c r="F395" s="32" t="n"/>
-    </row>
-    <row r="396">
-      <c r="E396" s="29" t="n"/>
-      <c r="F396" s="32" t="n"/>
-    </row>
-    <row r="397">
-      <c r="E397" s="29" t="n"/>
-      <c r="F397" s="32" t="n"/>
-    </row>
-    <row r="398">
-      <c r="E398" s="29" t="n"/>
-      <c r="F398" s="32" t="n"/>
-    </row>
-    <row r="399">
-      <c r="E399" s="29" t="n"/>
-      <c r="F399" s="32" t="n"/>
-    </row>
-    <row r="400">
-      <c r="E400" s="29" t="n"/>
-      <c r="F400" s="32" t="n"/>
-    </row>
-    <row r="401">
-      <c r="E401" s="29" t="n"/>
-      <c r="F401" s="32" t="n"/>
-    </row>
-    <row r="402">
-      <c r="E402" s="29" t="n"/>
-      <c r="F402" s="32" t="n"/>
-    </row>
-    <row r="403">
-      <c r="E403" s="29" t="n"/>
-      <c r="F403" s="32" t="n"/>
-    </row>
-    <row r="404">
-      <c r="E404" s="29" t="n"/>
-      <c r="F404" s="32" t="n"/>
-    </row>
-    <row r="405">
-      <c r="E405" s="29" t="n"/>
-      <c r="F405" s="32" t="n"/>
-    </row>
-    <row r="406">
-      <c r="E406" s="29" t="n"/>
-      <c r="F406" s="32" t="n"/>
-    </row>
-    <row r="407">
-      <c r="E407" s="29" t="n"/>
-      <c r="F407" s="32" t="n"/>
-    </row>
-    <row r="408">
-      <c r="E408" s="29" t="n"/>
-      <c r="F408" s="32" t="n"/>
-    </row>
-    <row r="409">
-      <c r="E409" s="29" t="n"/>
-      <c r="F409" s="32" t="n"/>
-    </row>
-    <row r="410">
-      <c r="E410" s="29" t="n"/>
-      <c r="F410" s="32" t="n"/>
-    </row>
-    <row r="411">
-      <c r="E411" s="29" t="n"/>
-      <c r="F411" s="32" t="n"/>
-    </row>
-    <row r="412">
-      <c r="E412" s="29" t="n"/>
-      <c r="F412" s="32" t="n"/>
-    </row>
-    <row r="413">
-      <c r="E413" s="29" t="n"/>
-      <c r="F413" s="32" t="n"/>
-    </row>
-    <row r="414">
-      <c r="E414" s="29" t="n"/>
-      <c r="F414" s="32" t="n"/>
-    </row>
-    <row r="415">
-      <c r="E415" s="29" t="n"/>
-      <c r="F415" s="32" t="n"/>
-    </row>
-    <row r="416">
-      <c r="E416" s="29" t="n"/>
-      <c r="F416" s="32" t="n"/>
-    </row>
-    <row r="417">
-      <c r="E417" s="29" t="n"/>
-      <c r="F417" s="32" t="n"/>
-    </row>
-    <row r="418">
-      <c r="E418" s="29" t="n"/>
-      <c r="F418" s="32" t="n"/>
-    </row>
-    <row r="419">
-      <c r="E419" s="29" t="n"/>
-      <c r="F419" s="32" t="n"/>
-    </row>
-    <row r="420">
-      <c r="E420" s="29" t="n"/>
-      <c r="F420" s="32" t="n"/>
-    </row>
-    <row r="421">
-      <c r="E421" s="29" t="n"/>
-      <c r="F421" s="32" t="n"/>
-    </row>
-    <row r="422">
-      <c r="E422" s="29" t="n"/>
-      <c r="F422" s="32" t="n"/>
-    </row>
-    <row r="423">
-      <c r="E423" s="29" t="n"/>
-      <c r="F423" s="32" t="n"/>
-    </row>
-    <row r="424">
-      <c r="E424" s="29" t="n"/>
-      <c r="F424" s="32" t="n"/>
-    </row>
-    <row r="425">
-      <c r="E425" s="29" t="n"/>
-      <c r="F425" s="32" t="n"/>
-    </row>
-    <row r="426">
-      <c r="E426" s="29" t="n"/>
-      <c r="F426" s="32" t="n"/>
-    </row>
-    <row r="427">
-      <c r="E427" s="29" t="n"/>
-      <c r="F427" s="32" t="n"/>
-    </row>
-    <row r="428">
-      <c r="E428" s="29" t="n"/>
-      <c r="F428" s="32" t="n"/>
-    </row>
-    <row r="429">
-      <c r="E429" s="29" t="n"/>
-      <c r="F429" s="32" t="n"/>
-    </row>
-    <row r="430">
-      <c r="E430" s="29" t="n"/>
-      <c r="F430" s="32" t="n"/>
-    </row>
-    <row r="431">
-      <c r="E431" s="29" t="n"/>
-      <c r="F431" s="32" t="n"/>
-    </row>
-    <row r="432">
-      <c r="E432" s="29" t="n"/>
-      <c r="F432" s="32" t="n"/>
-    </row>
-    <row r="433">
-      <c r="E433" s="29" t="n"/>
-      <c r="F433" s="32" t="n"/>
-    </row>
-    <row r="434">
-      <c r="E434" s="29" t="n"/>
-      <c r="F434" s="32" t="n"/>
-    </row>
-    <row r="435">
-      <c r="E435" s="29" t="n"/>
-      <c r="F435" s="32" t="n"/>
-    </row>
-    <row r="436">
-      <c r="E436" s="29" t="n"/>
-      <c r="F436" s="32" t="n"/>
-    </row>
-    <row r="437">
-      <c r="E437" s="29" t="n"/>
-      <c r="F437" s="32" t="n"/>
-    </row>
-    <row r="438">
-      <c r="E438" s="29" t="n"/>
-      <c r="F438" s="32" t="n"/>
-    </row>
-    <row r="439">
-      <c r="E439" s="29" t="n"/>
-      <c r="F439" s="32" t="n"/>
-    </row>
-    <row r="440">
-      <c r="E440" s="29" t="n"/>
-      <c r="F440" s="32" t="n"/>
-    </row>
-    <row r="441">
-      <c r="E441" s="29" t="n"/>
-      <c r="F441" s="32" t="n"/>
-    </row>
-    <row r="442">
-      <c r="E442" s="29" t="n"/>
-      <c r="F442" s="32" t="n"/>
-    </row>
-    <row r="443">
-      <c r="E443" s="29" t="n"/>
-      <c r="F443" s="32" t="n"/>
-    </row>
-    <row r="444">
-      <c r="E444" s="29" t="n"/>
-      <c r="F444" s="32" t="n"/>
-    </row>
-    <row r="445">
-      <c r="E445" s="29" t="n"/>
-      <c r="F445" s="32" t="n"/>
-    </row>
-    <row r="446">
-      <c r="E446" s="29" t="n"/>
-      <c r="F446" s="32" t="n"/>
-    </row>
-    <row r="447">
-      <c r="E447" s="29" t="n"/>
-      <c r="F447" s="32" t="n"/>
-    </row>
-    <row r="448">
-      <c r="E448" s="29" t="n"/>
-      <c r="F448" s="32" t="n"/>
-    </row>
-    <row r="449">
-      <c r="E449" s="29" t="n"/>
-      <c r="F449" s="32" t="n"/>
-    </row>
-    <row r="450">
-      <c r="E450" s="29" t="n"/>
-      <c r="F450" s="32" t="n"/>
-    </row>
-    <row r="451">
-      <c r="E451" s="29" t="n"/>
-      <c r="F451" s="32" t="n"/>
-    </row>
-    <row r="452">
-      <c r="E452" s="29" t="n"/>
-      <c r="F452" s="32" t="n"/>
-    </row>
-    <row r="453">
-      <c r="E453" s="29" t="n"/>
-      <c r="F453" s="32" t="n"/>
-    </row>
-    <row r="454">
-      <c r="E454" s="29" t="n"/>
-      <c r="F454" s="32" t="n"/>
-    </row>
-    <row r="455">
-      <c r="E455" s="29" t="n"/>
-      <c r="F455" s="32" t="n"/>
-    </row>
-    <row r="456">
-      <c r="E456" s="29" t="n"/>
-      <c r="F456" s="32" t="n"/>
-    </row>
-    <row r="457">
-      <c r="E457" s="29" t="n"/>
-      <c r="F457" s="32" t="n"/>
-    </row>
-    <row r="458">
-      <c r="E458" s="29" t="n"/>
-      <c r="F458" s="32" t="n"/>
-    </row>
-    <row r="459">
-      <c r="E459" s="29" t="n"/>
-      <c r="F459" s="32" t="n"/>
-    </row>
-    <row r="460">
-      <c r="E460" s="29" t="n"/>
-      <c r="F460" s="32" t="n"/>
-    </row>
-    <row r="461">
-      <c r="E461" s="29" t="n"/>
-      <c r="F461" s="32" t="n"/>
-    </row>
-    <row r="462">
-      <c r="E462" s="29" t="n"/>
-      <c r="F462" s="32" t="n"/>
-    </row>
-    <row r="463">
-      <c r="E463" s="29" t="n"/>
-      <c r="F463" s="32" t="n"/>
-    </row>
-    <row r="464">
-      <c r="E464" s="29" t="n"/>
-      <c r="F464" s="32" t="n"/>
-    </row>
-    <row r="465">
-      <c r="E465" s="29" t="n"/>
-      <c r="F465" s="32" t="n"/>
-    </row>
-    <row r="466">
-      <c r="E466" s="29" t="n"/>
-      <c r="F466" s="32" t="n"/>
-    </row>
-    <row r="467">
-      <c r="E467" s="29" t="n"/>
-      <c r="F467" s="32" t="n"/>
-    </row>
-    <row r="468">
-      <c r="E468" s="29" t="n"/>
-      <c r="F468" s="32" t="n"/>
-    </row>
-    <row r="469">
-      <c r="E469" s="29" t="n"/>
-      <c r="F469" s="32" t="n"/>
-    </row>
-    <row r="470">
-      <c r="E470" s="29" t="n"/>
-      <c r="F470" s="32" t="n"/>
-    </row>
-    <row r="471">
-      <c r="E471" s="29" t="n"/>
-      <c r="F471" s="32" t="n"/>
-    </row>
-    <row r="472">
-      <c r="E472" s="29" t="n"/>
-      <c r="F472" s="32" t="n"/>
-    </row>
-    <row r="473">
-      <c r="E473" s="29" t="n"/>
-      <c r="F473" s="32" t="n"/>
-    </row>
-    <row r="474">
-      <c r="E474" s="29" t="n"/>
-      <c r="F474" s="32" t="n"/>
-    </row>
-    <row r="475">
-      <c r="E475" s="29" t="n"/>
-      <c r="F475" s="32" t="n"/>
-    </row>
-    <row r="476">
-      <c r="E476" s="29" t="n"/>
-      <c r="F476" s="32" t="n"/>
-    </row>
-    <row r="477">
-      <c r="E477" s="29" t="n"/>
-      <c r="F477" s="32" t="n"/>
-    </row>
-    <row r="478">
-      <c r="E478" s="29" t="n"/>
-      <c r="F478" s="32" t="n"/>
-    </row>
-    <row r="479">
-      <c r="E479" s="29" t="n"/>
-      <c r="F479" s="32" t="n"/>
-    </row>
-    <row r="480">
-      <c r="E480" s="29" t="n"/>
-      <c r="F480" s="32" t="n"/>
-    </row>
-    <row r="481">
-      <c r="E481" s="29" t="n"/>
-      <c r="F481" s="32" t="n"/>
-    </row>
-    <row r="482">
-      <c r="E482" s="29" t="n"/>
-      <c r="F482" s="32" t="n"/>
-    </row>
-    <row r="483">
-      <c r="E483" s="29" t="n"/>
-      <c r="F483" s="32" t="n"/>
-    </row>
-    <row r="484">
-      <c r="E484" s="29" t="n"/>
-      <c r="F484" s="32" t="n"/>
-    </row>
-    <row r="485">
-      <c r="E485" s="29" t="n"/>
-      <c r="F485" s="32" t="n"/>
-    </row>
-    <row r="486">
-      <c r="E486" s="29" t="n"/>
-      <c r="F486" s="32" t="n"/>
-    </row>
-    <row r="487">
-      <c r="E487" s="29" t="n"/>
-      <c r="F487" s="32" t="n"/>
-    </row>
-    <row r="488">
-      <c r="E488" s="29" t="n"/>
-      <c r="F488" s="32" t="n"/>
-    </row>
-    <row r="489">
-      <c r="E489" s="29" t="n"/>
-      <c r="F489" s="32" t="n"/>
-    </row>
-    <row r="490">
-      <c r="E490" s="29" t="n"/>
-      <c r="F490" s="32" t="n"/>
-    </row>
-    <row r="491">
-      <c r="E491" s="29" t="n"/>
-      <c r="F491" s="32" t="n"/>
-    </row>
-    <row r="492">
-      <c r="E492" s="29" t="n"/>
-      <c r="F492" s="32" t="n"/>
-    </row>
-    <row r="493">
-      <c r="E493" s="29" t="n"/>
-      <c r="F493" s="32" t="n"/>
-    </row>
-    <row r="494">
-      <c r="E494" s="29" t="n"/>
-      <c r="F494" s="32" t="n"/>
-    </row>
-    <row r="495">
-      <c r="E495" s="29" t="n"/>
-      <c r="F495" s="32" t="n"/>
-    </row>
-    <row r="496">
-      <c r="E496" s="29" t="n"/>
-      <c r="F496" s="32" t="n"/>
-    </row>
-    <row r="497">
-      <c r="E497" s="29" t="n"/>
-      <c r="F497" s="32" t="n"/>
-    </row>
-    <row r="498">
-      <c r="E498" s="29" t="n"/>
-      <c r="F498" s="32" t="n"/>
-    </row>
-    <row r="499">
-      <c r="E499" s="29" t="n"/>
-      <c r="F499" s="32" t="n"/>
-    </row>
-    <row r="500">
-      <c r="E500" s="29" t="n"/>
-      <c r="F500" s="32" t="n"/>
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Несущие стены и перемычки</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Вывоз мусора с объекта</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>маш</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>10000</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>Перенесено из rows_to_add, статус: needs_review. Добавлено из калькулятора MVP, требуется проверка Елены Требуется проверка Елены.</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>waste_removal_truck</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11845,7 +12437,6 @@
           <t>15000</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -11883,7 +12474,6 @@
           <t>20000.000000</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -11921,7 +12511,6 @@
           <t>350</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -11959,7 +12548,6 @@
           <t>340</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -11997,7 +12585,6 @@
           <t>28000</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -12035,7 +12622,6 @@
           <t>15000</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -12073,7 +12659,6 @@
           <t>350</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -12111,7 +12696,6 @@
           <t>650</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -12149,7 +12733,6 @@
           <t>6400.000000</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -12187,7 +12770,6 @@
           <t>7500.000000</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -12225,7 +12807,6 @@
           <t>12000.000000</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -12263,7 +12844,6 @@
           <t>38000.000000</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -12301,7 +12881,6 @@
           <t>30000.000000</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -12339,7 +12918,6 @@
           <t>250</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -12377,7 +12955,6 @@
           <t>450.000000</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -12415,7 +12992,6 @@
           <t>900.000000</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -12453,7 +13029,6 @@
           <t>250</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -12491,7 +13066,6 @@
           <t>9020.000000</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -12529,7 +13103,6 @@
           <t>500</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -12567,7 +13140,6 @@
           <t>22000</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -12605,7 +13177,6 @@
           <t>9759.080000</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -12643,7 +13214,6 @@
           <t>20000.000000</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -12676,8 +13246,6 @@
           <t>м2</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -12715,7 +13283,6 @@
           <t>600.000000</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -12753,7 +13320,6 @@
           <t>1200</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -12791,7 +13357,6 @@
           <t>6000</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -12829,7 +13394,6 @@
           <t>5600</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -12867,7 +13431,6 @@
           <t>5500</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -12905,7 +13468,6 @@
           <t>7000</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -12943,7 +13505,6 @@
           <t>35</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -12981,7 +13542,6 @@
           <t>1000</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -13019,7 +13579,6 @@
           <t>5000</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -13057,7 +13616,6 @@
           <t>1200</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -13095,7 +13653,6 @@
           <t>22000.000000</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -13133,7 +13690,6 @@
           <t>100</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -13171,7 +13727,6 @@
           <t>1450.000000</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -13209,7 +13764,6 @@
           <t>98</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -13247,7 +13801,6 @@
           <t>95</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -13285,7 +13838,6 @@
           <t>30000</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -13323,7 +13875,6 @@
           <t>7326.7</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -13361,7 +13912,6 @@
           <t>6906.7</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -13399,7 +13949,6 @@
           <t>10896</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -13437,7 +13986,6 @@
           <t>10896</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -13475,7 +14023,6 @@
           <t>10896</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -13513,7 +14060,6 @@
           <t>10896</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -13551,7 +14097,6 @@
           <t>64.34</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -13589,7 +14134,6 @@
           <t>111.76</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -13627,7 +14171,6 @@
           <t>2500</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -13665,7 +14208,6 @@
           <t>5000</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -13703,7 +14245,6 @@
           <t>5000</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -13741,7 +14282,6 @@
           <t>51431</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -13779,7 +14319,6 @@
           <t>375</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -13817,7 +14356,6 @@
           <t>1200</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -13855,7 +14393,6 @@
           <t>1000</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -13888,8 +14425,6 @@
           <t>м3</t>
         </is>
       </c>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -13927,7 +14462,6 @@
           <t>20000</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -13965,7 +14499,6 @@
           <t>15000</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -14003,7 +14536,6 @@
           <t>5000.000000</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -14041,7 +14573,6 @@
           <t>100</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -14074,8 +14605,6 @@
           <t>м2</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr"/>
-      <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -14113,7 +14642,6 @@
           <t>21499.997319</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -14151,7 +14679,6 @@
           <t>400</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>
@@ -14189,7 +14716,6 @@
           <t>10000</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
         <is>
           <t>Добавлено из калькулятора MVP, требуется проверка Елены</t>

</xml_diff>

<commit_message>
fix(pricing): map Ø20 rebar price_code; add groove-lintel + foundation-wall schema fields
Price registry: rebar_a500_d20_m row had a real price but no price_code, so it
was invisible to both registry readers (which skip codeless rows) — mapped it
and confirmed all templated registry_code patterns in the system (rebar,
roof-slope) are now fully covered.

Extraction schema (diagnostic-only, no calculator.py changes): added the
groove-reinforced lintel type (floor_1/2_lintel_groove_length +
lintel_groove_rebar_items, kept separate from the calculator-wired
lintel_rebar_items to avoid its strict component validation) and
foundation_wall_items[]/column_footing_items[] repeated groups, per
UNIVERSALIZATION_PLAN.md P1. Verified via build_review_workbook_from_contracts.py.
</commit_message>
<xml_diff>
--- a/output/price_registry_filled_v3.xlsx
+++ b/output/price_registry_filled_v3.xlsx
@@ -3848,7 +3848,6 @@
           <t>price_code проставлен автоматически по точному совпадению номенклатуры; проверьте цену/единицу. Каталожная/поставщическая позиция. price_code не проставлен автоматически, если нет однозначной связи с текущей строкой калькулятора.</t>
         </is>
       </c>
-      <c r="H83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4414,7 +4413,12 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>price_code пока не сопоставлен; требуется ручная проверка связи с калькулятором.</t>
+          <t>price_code сопоставлен 2026-07-20 (rebar_a500_d20_m), проверено связью с калькулятором floor_slab_2/floor_slab_1.</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>rebar_a500_d20_m</t>
         </is>
       </c>
     </row>
@@ -4901,7 +4905,6 @@
           <t>price_code проставлен автоматически по точному совпадению номенклатуры; проверьте цену/единицу. Позиция кровельного прайса. price_code не проставлен автоматически, если текущие калькуляторы пока не используют эту строку напрямую.</t>
         </is>
       </c>
-      <c r="H117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">

</xml_diff>